<commit_message>
Agregando ganancias y perdidas totales en general para tener un paneo de perdidas/ganancias totales sumadas de todas las monedas
</commit_message>
<xml_diff>
--- a/operaciones_crypto2.xlsx
+++ b/operaciones_crypto2.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -497,17 +497,17 @@
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
+          <t>0.04948046</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H2" s="1" t="inlineStr">
-        <is>
-          <t>0.04948046</t>
-        </is>
-      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>CERRADA</t>
         </is>
       </c>
     </row>
@@ -989,17 +989,17 @@
       </c>
       <c r="G14" s="1" t="inlineStr">
         <is>
+          <t>55.61735261</t>
+        </is>
+      </c>
+      <c r="H14" s="1" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H14" s="1" t="inlineStr">
-        <is>
-          <t>55.61735261</t>
-        </is>
-      </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>CERRADA</t>
         </is>
       </c>
     </row>
@@ -1112,17 +1112,17 @@
       </c>
       <c r="G17" s="1" t="inlineStr">
         <is>
+          <t>0.00077259</t>
+        </is>
+      </c>
+      <c r="H17" s="1" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H17" s="1" t="inlineStr">
-        <is>
-          <t>0.00077259</t>
-        </is>
-      </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>CERRADA</t>
         </is>
       </c>
     </row>
@@ -1235,17 +1235,17 @@
       </c>
       <c r="G20" s="1" t="inlineStr">
         <is>
+          <t>0.00084752</t>
+        </is>
+      </c>
+      <c r="H20" s="1" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H20" s="1" t="inlineStr">
-        <is>
-          <t>0.00084752</t>
-        </is>
-      </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>CERRADA</t>
         </is>
       </c>
     </row>
@@ -1399,17 +1399,17 @@
       </c>
       <c r="G24" s="1" t="inlineStr">
         <is>
+          <t>868.05555556</t>
+        </is>
+      </c>
+      <c r="H24" s="1" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H24" s="1" t="inlineStr">
-        <is>
-          <t>868.05555556</t>
-        </is>
-      </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>CERRADA</t>
         </is>
       </c>
     </row>
@@ -1440,15 +1440,179 @@
       </c>
       <c r="G25" s="1" t="inlineStr">
         <is>
+          <t>51.44032922</t>
+        </is>
+      </c>
+      <c r="H25" s="1" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H25" s="1" t="inlineStr">
-        <is>
-          <t>51.44032922</t>
-        </is>
-      </c>
       <c r="I25" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>axs</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>5-08-2026</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>50</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.867</v>
+      </c>
+      <c r="F26" s="1" t="inlineStr">
+        <is>
+          <t>57.67012687</t>
+        </is>
+      </c>
+      <c r="G26" s="1" t="inlineStr">
+        <is>
+          <t>57.67012687</t>
+        </is>
+      </c>
+      <c r="H26" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>dot</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>14-08-2026</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>50</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.761</v>
+      </c>
+      <c r="F27" s="1" t="inlineStr">
+        <is>
+          <t>65.70302234</t>
+        </is>
+      </c>
+      <c r="G27" s="1" t="inlineStr">
+        <is>
+          <t>65.70302234</t>
+        </is>
+      </c>
+      <c r="H27" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>axs</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>1-09-2026</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>50</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.9350000000000001</v>
+      </c>
+      <c r="F28" s="1" t="inlineStr">
+        <is>
+          <t>53.47593583</t>
+        </is>
+      </c>
+      <c r="G28" s="1" t="inlineStr">
+        <is>
+          <t>53.47593583</t>
+        </is>
+      </c>
+      <c r="H28" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ron</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>19-09-2026</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>50</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.0473</v>
+      </c>
+      <c r="F29" s="1" t="inlineStr">
+        <is>
+          <t>1057.08245243</t>
+        </is>
+      </c>
+      <c r="G29" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H29" s="1" t="inlineStr">
+        <is>
+          <t>1057.08245243</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
         <is>
           <t>ABIERTA</t>
         </is>
@@ -1465,7 +1629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2073,6 +2237,321 @@
       </c>
       <c r="I17" t="n">
         <v>4.888580694717071</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="n">
+        <v>16</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>btc</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>16-07-2026</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t>0.00077259</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>64680</v>
+      </c>
+      <c r="G18" t="n">
+        <v>49.9711212</v>
+      </c>
+      <c r="H18" t="n">
+        <v>46</v>
+      </c>
+      <c r="I18" t="n">
+        <v>3.971121199999999</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="n">
+        <v>19</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>btc</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>16-07-2026</t>
+        </is>
+      </c>
+      <c r="E19" s="1" t="inlineStr">
+        <is>
+          <t>0.00084752</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>64680</v>
+      </c>
+      <c r="G19" t="n">
+        <v>54.8175936</v>
+      </c>
+      <c r="H19" t="n">
+        <v>50</v>
+      </c>
+      <c r="I19" t="n">
+        <v>4.817593600000002</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="n">
+        <v>25</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>axs</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>19-08-2026</t>
+        </is>
+      </c>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t>57.67012687</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>0.902</v>
+      </c>
+      <c r="G20" t="n">
+        <v>52.01845443674</v>
+      </c>
+      <c r="H20" t="n">
+        <v>50</v>
+      </c>
+      <c r="I20" t="n">
+        <v>2.018454436740001</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>eth</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>19-08-2026</t>
+        </is>
+      </c>
+      <c r="E21" s="1" t="inlineStr">
+        <is>
+          <t>0.04948046</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>2126</v>
+      </c>
+      <c r="G21" t="n">
+        <v>105.19545796</v>
+      </c>
+      <c r="H21" t="n">
+        <v>100</v>
+      </c>
+      <c r="I21" t="n">
+        <v>5.195457959999999</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="n">
+        <v>26</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>dot</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>20-08-2026</t>
+        </is>
+      </c>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>65.70302234</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>0.838</v>
+      </c>
+      <c r="G22" t="n">
+        <v>55.05913272092</v>
+      </c>
+      <c r="H22" t="n">
+        <v>50</v>
+      </c>
+      <c r="I22" t="n">
+        <v>5.059132720920005</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="n">
+        <v>23</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ronin</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>21-08-2026</t>
+        </is>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>868.05555556</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>0.0586</v>
+      </c>
+      <c r="G23" t="n">
+        <v>50.868055555816</v>
+      </c>
+      <c r="H23" t="n">
+        <v>50</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.8680555558159995</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="n">
+        <v>24</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>axs</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>22-08-2026</t>
+        </is>
+      </c>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t>51.44032922</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>1.092</v>
+      </c>
+      <c r="G24" t="n">
+        <v>56.17283950824001</v>
+      </c>
+      <c r="H24" t="n">
+        <v>50</v>
+      </c>
+      <c r="I24" t="n">
+        <v>6.17283950824001</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="n">
+        <v>13</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>dot</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>22-08-2026</t>
+        </is>
+      </c>
+      <c r="E25" s="1" t="inlineStr">
+        <is>
+          <t>55.61735261</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>1.018</v>
+      </c>
+      <c r="G25" t="n">
+        <v>56.61846495698</v>
+      </c>
+      <c r="H25" t="n">
+        <v>50</v>
+      </c>
+      <c r="I25" t="n">
+        <v>6.618464956979999</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="n">
+        <v>27</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>axs</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>18-09-2026</t>
+        </is>
+      </c>
+      <c r="E26" s="1" t="inlineStr">
+        <is>
+          <t>53.47593583</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>1.019</v>
+      </c>
+      <c r="G26" t="n">
+        <v>54.49197861076999</v>
+      </c>
+      <c r="H26" t="n">
+        <v>50</v>
+      </c>
+      <c r="I26" t="n">
+        <v>4.491978610769991</v>
       </c>
     </row>
   </sheetData>
@@ -2086,7 +2565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2138,27 +2617,27 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>eth</t>
+          <t>ronin</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>23-05-2026</t>
+          <t>22-05-2026</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="E2" t="n">
-        <v>2021</v>
+        <v>0.0936</v>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>0.04948046</t>
+          <t>534.18803419</t>
         </is>
       </c>
       <c r="G2" s="1" t="inlineStr">
@@ -2168,7 +2647,7 @@
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t>0.04948046</t>
+          <t>534.18803419</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -2179,7 +2658,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -2188,18 +2667,18 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>22-05-2026</t>
+          <t>30-05-2026</t>
         </is>
       </c>
       <c r="D3" t="n">
         <v>50</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0936</v>
+        <v>0.0785</v>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>534.18803419</t>
+          <t>636.94267516</t>
         </is>
       </c>
       <c r="G3" s="1" t="inlineStr">
@@ -2209,7 +2688,7 @@
       </c>
       <c r="H3" s="1" t="inlineStr">
         <is>
-          <t>534.18803419</t>
+          <t>636.94267516</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -2220,7 +2699,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -2229,18 +2708,18 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>30-05-2026</t>
+          <t>23-06-2026</t>
         </is>
       </c>
       <c r="D4" t="n">
         <v>50</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0785</v>
+        <v>0.0591</v>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>636.94267516</t>
+          <t>846.02368866</t>
         </is>
       </c>
       <c r="G4" s="1" t="inlineStr">
@@ -2250,7 +2729,7 @@
       </c>
       <c r="H4" s="1" t="inlineStr">
         <is>
-          <t>636.94267516</t>
+          <t>846.02368866</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -2261,27 +2740,27 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ronin</t>
+          <t>ron</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>23-06-2026</t>
+          <t>19-09-2026</t>
         </is>
       </c>
       <c r="D5" t="n">
         <v>50</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0591</v>
+        <v>0.0473</v>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>846.02368866</t>
+          <t>1057.08245243</t>
         </is>
       </c>
       <c r="G5" s="1" t="inlineStr">
@@ -2291,215 +2770,10 @@
       </c>
       <c r="H5" s="1" t="inlineStr">
         <is>
-          <t>846.02368866</t>
+          <t>1057.08245243</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
-        <is>
-          <t>ABIERTA</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>13</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>dot</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>23-06-2026</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>50</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0.899</v>
-      </c>
-      <c r="F6" s="1" t="inlineStr">
-        <is>
-          <t>55.61735261</t>
-        </is>
-      </c>
-      <c r="G6" s="1" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H6" s="1" t="inlineStr">
-        <is>
-          <t>55.61735261</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>ABIERTA</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>16</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>btc</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>28-06-2026</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>46</v>
-      </c>
-      <c r="E7" t="n">
-        <v>59540</v>
-      </c>
-      <c r="F7" s="1" t="inlineStr">
-        <is>
-          <t>0.00077259</t>
-        </is>
-      </c>
-      <c r="G7" s="1" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H7" s="1" t="inlineStr">
-        <is>
-          <t>0.00077259</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>ABIERTA</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>19</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>btc</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>30-06-2026</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>50</v>
-      </c>
-      <c r="E8" t="n">
-        <v>58996</v>
-      </c>
-      <c r="F8" s="1" t="inlineStr">
-        <is>
-          <t>0.00084752</t>
-        </is>
-      </c>
-      <c r="G8" s="1" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H8" s="1" t="inlineStr">
-        <is>
-          <t>0.00084752</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>ABIERTA</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>23</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>ronin</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>7-7-2026</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>50</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0.0576</v>
-      </c>
-      <c r="F9" s="1" t="inlineStr">
-        <is>
-          <t>868.05555556</t>
-        </is>
-      </c>
-      <c r="G9" s="1" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H9" s="1" t="inlineStr">
-        <is>
-          <t>868.05555556</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>ABIERTA</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>24</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>axs</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>08-07-2026</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>50</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0.972</v>
-      </c>
-      <c r="F10" s="1" t="inlineStr">
-        <is>
-          <t>51.44032922</t>
-        </is>
-      </c>
-      <c r="G10" s="1" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H10" s="1" t="inlineStr">
-        <is>
-          <t>51.44032922</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
         <is>
           <t>ABIERTA</t>
         </is>
@@ -2516,7 +2790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2593,7 +2867,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -2602,34 +2876,34 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>23-05-2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>15-06-2026</t>
+          <t>19-08-2026</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>110.6542056074766</v>
+        <v>105.19545796</v>
       </c>
       <c r="G2" t="n">
-        <v>1605</v>
+        <v>2021</v>
       </c>
       <c r="H2" t="n">
-        <v>1776</v>
+        <v>2126</v>
       </c>
       <c r="I2" s="1" t="inlineStr">
         <is>
-          <t>0.12461059</t>
+          <t>0.04948046</t>
         </is>
       </c>
       <c r="J2" s="1" t="inlineStr">
         <is>
-          <t>0.12461059</t>
+          <t>0.04948046</t>
         </is>
       </c>
       <c r="K2" s="1" t="inlineStr">
@@ -2641,7 +2915,7 @@
         <v>100</v>
       </c>
       <c r="M2" t="n">
-        <v>10.65420560747661</v>
+        <v>5.195457959999999</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -2672,13 +2946,13 @@
         <v>200</v>
       </c>
       <c r="F3" t="n">
-        <v>113.1464174454828</v>
+        <v>110.6542056074766</v>
       </c>
       <c r="G3" t="n">
         <v>1605</v>
       </c>
       <c r="H3" t="n">
-        <v>1816</v>
+        <v>1776</v>
       </c>
       <c r="I3" s="1" t="inlineStr">
         <is>
@@ -2699,7 +2973,7 @@
         <v>100</v>
       </c>
       <c r="M3" t="n">
-        <v>13.14641744548284</v>
+        <v>10.65420560747661</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -2709,7 +2983,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -2723,29 +2997,29 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>14-06-2026</t>
+          <t>15-06-2026</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="F4" t="n">
-        <v>109.7514340344168</v>
+        <v>113.1464174454828</v>
       </c>
       <c r="G4" t="n">
-        <v>1569</v>
+        <v>1605</v>
       </c>
       <c r="H4" t="n">
-        <v>1722</v>
+        <v>1816</v>
       </c>
       <c r="I4" s="1" t="inlineStr">
         <is>
-          <t>0.06373486</t>
+          <t>0.12461059</t>
         </is>
       </c>
       <c r="J4" s="1" t="inlineStr">
         <is>
-          <t>0.06373486</t>
+          <t>0.12461059</t>
         </is>
       </c>
       <c r="K4" s="1" t="inlineStr">
@@ -2757,7 +3031,7 @@
         <v>100</v>
       </c>
       <c r="M4" t="n">
-        <v>9.751434034416832</v>
+        <v>13.14641744548284</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -2767,7 +3041,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -2776,34 +3050,34 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>06-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>07-06-2026</t>
+          <t>14-06-2026</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F5" t="n">
-        <v>55.23560209424085</v>
+        <v>109.7514340344168</v>
       </c>
       <c r="G5" t="n">
-        <v>1528</v>
+        <v>1569</v>
       </c>
       <c r="H5" t="n">
-        <v>1688</v>
+        <v>1722</v>
       </c>
       <c r="I5" s="1" t="inlineStr">
         <is>
-          <t>0.03272251</t>
+          <t>0.06373486</t>
         </is>
       </c>
       <c r="J5" s="1" t="inlineStr">
         <is>
-          <t>0.03272251</t>
+          <t>0.06373486</t>
         </is>
       </c>
       <c r="K5" s="1" t="inlineStr">
@@ -2812,10 +3086,10 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="M5" t="n">
-        <v>5.235602094240846</v>
+        <v>9.751434034416832</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -2825,11 +3099,11 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ronin</t>
+          <t>eth</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2839,29 +3113,29 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>07-06-2026</t>
         </is>
       </c>
       <c r="E6" t="n">
         <v>50</v>
       </c>
       <c r="F6" t="n">
-        <v>51.04166666666667</v>
+        <v>55.23560209424085</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0624</v>
+        <v>1528</v>
       </c>
       <c r="H6" t="n">
-        <v>0.06370000000000001</v>
+        <v>1688</v>
       </c>
       <c r="I6" s="1" t="inlineStr">
         <is>
-          <t>801.28205128</t>
+          <t>0.03272251</t>
         </is>
       </c>
       <c r="J6" s="1" t="inlineStr">
         <is>
-          <t>801.28205128</t>
+          <t>0.03272251</t>
         </is>
       </c>
       <c r="K6" s="1" t="inlineStr">
@@ -2873,7 +3147,7 @@
         <v>50</v>
       </c>
       <c r="M6" t="n">
-        <v>1.041666666666671</v>
+        <v>5.235602094240846</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -2883,43 +3157,43 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>uni</t>
+          <t>ronin</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>23-05-2026</t>
+          <t>06-06-2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>16-06-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F7" t="n">
-        <v>100.609198903442</v>
+        <v>51.04166666666667</v>
       </c>
       <c r="G7" t="n">
-        <v>3.283</v>
+        <v>0.0624</v>
       </c>
       <c r="H7" t="n">
-        <v>3.303</v>
+        <v>0.06370000000000001</v>
       </c>
       <c r="I7" s="1" t="inlineStr">
         <is>
-          <t>30.45994517</t>
+          <t>801.28205128</t>
         </is>
       </c>
       <c r="J7" s="1" t="inlineStr">
         <is>
-          <t>30.45994517</t>
+          <t>801.28205128</t>
         </is>
       </c>
       <c r="K7" s="1" t="inlineStr">
@@ -2928,10 +3202,10 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="M7" t="n">
-        <v>0.609198903441964</v>
+        <v>1.041666666666671</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -2941,7 +3215,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -2950,34 +3224,34 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>02-06-2026</t>
+          <t>23-05-2026</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>15-06-2026</t>
+          <t>16-06-2026</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="F8" t="n">
-        <v>64.57408732999284</v>
+        <v>100.609198903442</v>
       </c>
       <c r="G8" t="n">
-        <v>2.794</v>
+        <v>3.283</v>
       </c>
       <c r="H8" t="n">
-        <v>3.007</v>
+        <v>3.303</v>
       </c>
       <c r="I8" s="1" t="inlineStr">
         <is>
-          <t>21.4745884</t>
+          <t>30.45994517</t>
         </is>
       </c>
       <c r="J8" s="1" t="inlineStr">
         <is>
-          <t>21.4745884</t>
+          <t>30.45994517</t>
         </is>
       </c>
       <c r="K8" s="1" t="inlineStr">
@@ -2986,10 +3260,10 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>59.99999999999999</v>
+        <v>100</v>
       </c>
       <c r="M8" t="n">
-        <v>4.574087329992842</v>
+        <v>0.609198903441964</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
@@ -2999,7 +3273,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -3008,34 +3282,34 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>02-06-2026</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>14-06-2026</t>
+          <t>15-06-2026</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="F9" t="n">
-        <v>40.4636803874092</v>
+        <v>64.57408732999284</v>
       </c>
       <c r="G9" t="n">
-        <v>2.478</v>
+        <v>2.794</v>
       </c>
       <c r="H9" t="n">
-        <v>2.571</v>
+        <v>3.007</v>
       </c>
       <c r="I9" s="1" t="inlineStr">
         <is>
-          <t>15.73849879</t>
+          <t>21.4745884</t>
         </is>
       </c>
       <c r="J9" s="1" t="inlineStr">
         <is>
-          <t>15.73849879</t>
+          <t>21.4745884</t>
         </is>
       </c>
       <c r="K9" s="1" t="inlineStr">
@@ -3044,10 +3318,10 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>39</v>
+        <v>59.99999999999999</v>
       </c>
       <c r="M9" t="n">
-        <v>1.463680387409198</v>
+        <v>4.574087329992842</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -3057,7 +3331,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -3066,34 +3340,34 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>21-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10-07-2026</t>
+          <t>14-06-2026</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="F10" t="n">
-        <v>59.63347388906908</v>
+        <v>40.4636803874092</v>
       </c>
       <c r="G10" t="n">
-        <v>3.083</v>
+        <v>2.478</v>
       </c>
       <c r="H10" t="n">
-        <v>3.677</v>
+        <v>2.571</v>
       </c>
       <c r="I10" s="1" t="inlineStr">
         <is>
-          <t>16.21796951</t>
+          <t>15.73849879</t>
         </is>
       </c>
       <c r="J10" s="1" t="inlineStr">
         <is>
-          <t>16.21796951</t>
+          <t>15.73849879</t>
         </is>
       </c>
       <c r="K10" s="1" t="inlineStr">
@@ -3102,10 +3376,10 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="M10" t="n">
-        <v>9.63347388906908</v>
+        <v>1.463680387409198</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
@@ -3115,43 +3389,43 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>eth</t>
+          <t>uni</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>24-06-2026</t>
+          <t>21-06-2026</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>10-07-2026</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F11" t="n">
-        <v>112.6243059839605</v>
+        <v>59.63347388906908</v>
       </c>
       <c r="G11" t="n">
-        <v>1621</v>
+        <v>3.083</v>
       </c>
       <c r="H11" t="n">
-        <v>1825.64</v>
+        <v>3.677</v>
       </c>
       <c r="I11" s="1" t="inlineStr">
         <is>
-          <t>0.06169031</t>
+          <t>16.21796951</t>
         </is>
       </c>
       <c r="J11" s="1" t="inlineStr">
         <is>
-          <t>0.06169031</t>
+          <t>16.21796951</t>
         </is>
       </c>
       <c r="K11" s="1" t="inlineStr">
@@ -3160,10 +3434,10 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="M11" t="n">
-        <v>12.62430598396051</v>
+        <v>9.63347388906908</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
@@ -3173,43 +3447,43 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>eth</t>
+          <t>dot</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>23-06-2026</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10-07-2026</t>
+          <t>22-08-2026</t>
         </is>
       </c>
       <c r="E12" t="n">
         <v>50</v>
       </c>
       <c r="F12" t="n">
-        <v>56.86052463211772</v>
+        <v>56.61846495698</v>
       </c>
       <c r="G12" t="n">
-        <v>1563</v>
+        <v>0.899</v>
       </c>
       <c r="H12" t="n">
-        <v>1777.46</v>
+        <v>1.018</v>
       </c>
       <c r="I12" s="1" t="inlineStr">
         <is>
-          <t>0.03198976</t>
+          <t>55.61735261</t>
         </is>
       </c>
       <c r="J12" s="1" t="inlineStr">
         <is>
-          <t>0.03198976</t>
+          <t>55.61735261</t>
         </is>
       </c>
       <c r="K12" s="1" t="inlineStr">
@@ -3221,7 +3495,7 @@
         <v>50</v>
       </c>
       <c r="M12" t="n">
-        <v>6.860524632117723</v>
+        <v>6.618464956979999</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
@@ -3231,43 +3505,43 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>uni</t>
+          <t>eth</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>28-06-2026</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10-07-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F13" t="n">
-        <v>60.84024896265561</v>
+        <v>112.6243059839605</v>
       </c>
       <c r="G13" t="n">
-        <v>2.892</v>
+        <v>1621</v>
       </c>
       <c r="H13" t="n">
-        <v>3.519</v>
+        <v>1825.64</v>
       </c>
       <c r="I13" s="1" t="inlineStr">
         <is>
-          <t>17.28907331</t>
+          <t>0.06169031</t>
         </is>
       </c>
       <c r="J13" s="1" t="inlineStr">
         <is>
-          <t>17.28907331</t>
+          <t>0.06169031</t>
         </is>
       </c>
       <c r="K13" s="1" t="inlineStr">
@@ -3276,10 +3550,10 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="M13" t="n">
-        <v>10.84024896265561</v>
+        <v>12.62430598396051</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
@@ -3289,16 +3563,16 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>uni</t>
+          <t>eth</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>30-06-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -3310,22 +3584,22 @@
         <v>50</v>
       </c>
       <c r="F14" t="n">
-        <v>62.15183058147881</v>
+        <v>56.86052463211772</v>
       </c>
       <c r="G14" t="n">
-        <v>2.786</v>
+        <v>1563</v>
       </c>
       <c r="H14" t="n">
-        <v>3.4631</v>
+        <v>1777.46</v>
       </c>
       <c r="I14" s="1" t="inlineStr">
         <is>
-          <t>17.94687724</t>
+          <t>0.03198976</t>
         </is>
       </c>
       <c r="J14" s="1" t="inlineStr">
         <is>
-          <t>17.94687724</t>
+          <t>0.03198976</t>
         </is>
       </c>
       <c r="K14" s="1" t="inlineStr">
@@ -3337,7 +3611,7 @@
         <v>50</v>
       </c>
       <c r="M14" t="n">
-        <v>12.15183058147881</v>
+        <v>6.860524632117723</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -3347,43 +3621,43 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>eth</t>
+          <t>btc</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>30-06-2026</t>
+          <t>28-06-2026</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10-07-2026</t>
+          <t>16-07-2026</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="F15" t="n">
-        <v>56.42730158730157</v>
+        <v>49.9711212</v>
       </c>
       <c r="G15" t="n">
-        <v>1575</v>
+        <v>59540</v>
       </c>
       <c r="H15" t="n">
-        <v>1777.46</v>
+        <v>64680</v>
       </c>
       <c r="I15" s="1" t="inlineStr">
         <is>
-          <t>0.03174603</t>
+          <t>0.00077259</t>
         </is>
       </c>
       <c r="J15" s="1" t="inlineStr">
         <is>
-          <t>0.03174603</t>
+          <t>0.00077259</t>
         </is>
       </c>
       <c r="K15" s="1" t="inlineStr">
@@ -3392,10 +3666,10 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="M15" t="n">
-        <v>6.427301587301571</v>
+        <v>3.971121199999999</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
@@ -3405,43 +3679,43 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>btc</t>
+          <t>uni</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>30-06-2026</t>
+          <t>28-06-2026</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>10-07-2026</t>
         </is>
       </c>
       <c r="E16" t="n">
         <v>50</v>
       </c>
       <c r="F16" t="n">
-        <v>54.88858069471707</v>
+        <v>60.84024896265561</v>
       </c>
       <c r="G16" t="n">
-        <v>58585</v>
+        <v>2.892</v>
       </c>
       <c r="H16" t="n">
-        <v>64312.95</v>
+        <v>3.519</v>
       </c>
       <c r="I16" s="1" t="inlineStr">
         <is>
-          <t>0.00085346</t>
+          <t>17.28907331</t>
         </is>
       </c>
       <c r="J16" s="1" t="inlineStr">
         <is>
-          <t>0.00085346</t>
+          <t>17.28907331</t>
         </is>
       </c>
       <c r="K16" s="1" t="inlineStr">
@@ -3453,7 +3727,7 @@
         <v>50</v>
       </c>
       <c r="M16" t="n">
-        <v>4.888580694717071</v>
+        <v>10.84024896265561</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
@@ -3463,57 +3737,579 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
+        <v>18</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>uni</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>30-06-2026</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>10-07-2026</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>50</v>
+      </c>
+      <c r="F17" t="n">
+        <v>62.15183058147881</v>
+      </c>
+      <c r="G17" t="n">
+        <v>2.786</v>
+      </c>
+      <c r="H17" t="n">
+        <v>3.4631</v>
+      </c>
+      <c r="I17" s="1" t="inlineStr">
+        <is>
+          <t>17.94687724</t>
+        </is>
+      </c>
+      <c r="J17" s="1" t="inlineStr">
+        <is>
+          <t>17.94687724</t>
+        </is>
+      </c>
+      <c r="K17" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
+        <v>50</v>
+      </c>
+      <c r="M17" t="n">
+        <v>12.15183058147881</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>19</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>btc</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>30-06-2026</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>16-07-2026</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>50</v>
+      </c>
+      <c r="F18" t="n">
+        <v>54.8175936</v>
+      </c>
+      <c r="G18" t="n">
+        <v>58996</v>
+      </c>
+      <c r="H18" t="n">
+        <v>64680</v>
+      </c>
+      <c r="I18" s="1" t="inlineStr">
+        <is>
+          <t>0.00084752</t>
+        </is>
+      </c>
+      <c r="J18" s="1" t="inlineStr">
+        <is>
+          <t>0.00084752</t>
+        </is>
+      </c>
+      <c r="K18" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L18" t="n">
+        <v>50</v>
+      </c>
+      <c r="M18" t="n">
+        <v>4.817593600000002</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>20</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>eth</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>30-06-2026</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>10-07-2026</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>50</v>
+      </c>
+      <c r="F19" t="n">
+        <v>56.42730158730157</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1575</v>
+      </c>
+      <c r="H19" t="n">
+        <v>1777.46</v>
+      </c>
+      <c r="I19" s="1" t="inlineStr">
+        <is>
+          <t>0.03174603</t>
+        </is>
+      </c>
+      <c r="J19" s="1" t="inlineStr">
+        <is>
+          <t>0.03174603</t>
+        </is>
+      </c>
+      <c r="K19" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>50</v>
+      </c>
+      <c r="M19" t="n">
+        <v>6.427301587301571</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>21</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>btc</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>30-06-2026</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>11-07-2026</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>50</v>
+      </c>
+      <c r="F20" t="n">
+        <v>54.88858069471707</v>
+      </c>
+      <c r="G20" t="n">
+        <v>58585</v>
+      </c>
+      <c r="H20" t="n">
+        <v>64312.95</v>
+      </c>
+      <c r="I20" s="1" t="inlineStr">
+        <is>
+          <t>0.00085346</t>
+        </is>
+      </c>
+      <c r="J20" s="1" t="inlineStr">
+        <is>
+          <t>0.00085346</t>
+        </is>
+      </c>
+      <c r="K20" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
+        <v>50</v>
+      </c>
+      <c r="M20" t="n">
+        <v>4.888580694717071</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
         <v>22</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>ronin</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>30-06-2026</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>04-07-2026</t>
         </is>
       </c>
-      <c r="E17" t="n">
+      <c r="E21" t="n">
         <v>42</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F21" t="n">
         <v>47.067366</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G21" t="n">
         <v>0.0547</v>
       </c>
-      <c r="H17" t="n">
+      <c r="H21" t="n">
         <v>0.0613</v>
       </c>
-      <c r="I17" s="1" t="inlineStr">
+      <c r="I21" s="1" t="inlineStr">
         <is>
           <t>767.82449726</t>
         </is>
       </c>
-      <c r="J17" s="1" t="inlineStr">
+      <c r="J21" s="1" t="inlineStr">
         <is>
           <t>767.82449726</t>
         </is>
       </c>
-      <c r="K17" s="1" t="inlineStr">
+      <c r="K21" s="1" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L17" t="n">
+      <c r="L21" t="n">
         <v>41.999754</v>
       </c>
-      <c r="M17" t="n">
+      <c r="M21" t="n">
         <v>5.067611999999997</v>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>23</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ronin</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>7-7-2026</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>21-08-2026</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>50</v>
+      </c>
+      <c r="F22" t="n">
+        <v>50.868055555816</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.0576</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.0586</v>
+      </c>
+      <c r="I22" s="1" t="inlineStr">
+        <is>
+          <t>868.05555556</t>
+        </is>
+      </c>
+      <c r="J22" s="1" t="inlineStr">
+        <is>
+          <t>868.05555556</t>
+        </is>
+      </c>
+      <c r="K22" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L22" t="n">
+        <v>50</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0.8680555558159995</v>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>24</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>axs</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>08-07-2026</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>22-08-2026</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>50</v>
+      </c>
+      <c r="F23" t="n">
+        <v>56.17283950824001</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.972</v>
+      </c>
+      <c r="H23" t="n">
+        <v>1.092</v>
+      </c>
+      <c r="I23" s="1" t="inlineStr">
+        <is>
+          <t>51.44032922</t>
+        </is>
+      </c>
+      <c r="J23" s="1" t="inlineStr">
+        <is>
+          <t>51.44032922</t>
+        </is>
+      </c>
+      <c r="K23" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L23" t="n">
+        <v>50</v>
+      </c>
+      <c r="M23" t="n">
+        <v>6.17283950824001</v>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>25</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>axs</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>5-08-2026</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>19-08-2026</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>50</v>
+      </c>
+      <c r="F24" t="n">
+        <v>52.01845443674</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.867</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.902</v>
+      </c>
+      <c r="I24" s="1" t="inlineStr">
+        <is>
+          <t>57.67012687</t>
+        </is>
+      </c>
+      <c r="J24" s="1" t="inlineStr">
+        <is>
+          <t>57.67012687</t>
+        </is>
+      </c>
+      <c r="K24" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L24" t="n">
+        <v>50</v>
+      </c>
+      <c r="M24" t="n">
+        <v>2.018454436740001</v>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>26</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>dot</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>14-08-2026</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>20-08-2026</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>50</v>
+      </c>
+      <c r="F25" t="n">
+        <v>55.05913272092</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.761</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.838</v>
+      </c>
+      <c r="I25" s="1" t="inlineStr">
+        <is>
+          <t>65.70302234</t>
+        </is>
+      </c>
+      <c r="J25" s="1" t="inlineStr">
+        <is>
+          <t>65.70302234</t>
+        </is>
+      </c>
+      <c r="K25" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L25" t="n">
+        <v>50</v>
+      </c>
+      <c r="M25" t="n">
+        <v>5.059132720920005</v>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>27</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>axs</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1-09-2026</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>18-09-2026</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>50</v>
+      </c>
+      <c r="F26" t="n">
+        <v>54.49197861076999</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.9350000000000001</v>
+      </c>
+      <c r="H26" t="n">
+        <v>1.019</v>
+      </c>
+      <c r="I26" s="1" t="inlineStr">
+        <is>
+          <t>53.47593583</t>
+        </is>
+      </c>
+      <c r="J26" s="1" t="inlineStr">
+        <is>
+          <t>53.47593583</t>
+        </is>
+      </c>
+      <c r="K26" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L26" t="n">
+        <v>50</v>
+      </c>
+      <c r="M26" t="n">
+        <v>4.491978610769991</v>
+      </c>
+      <c r="N26" t="inlineStr">
         <is>
           <t>CERRADA</t>
         </is>
@@ -3530,7 +4326,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3567,16 +4363,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>64.69979138499693</v>
+        <v>69.89524934499693</v>
       </c>
       <c r="C2" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
@@ -3586,16 +4382,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6.109278666666668</v>
+        <v>6.977334222482668</v>
       </c>
       <c r="C3" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -3624,16 +4420,16 @@
         </is>
       </c>
       <c r="B5" t="n">
+        <v>11.6775976779</v>
+      </c>
+      <c r="C5" t="n">
         <v>0</v>
       </c>
-      <c r="C5" t="n">
-        <v>50</v>
-      </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -3643,16 +4439,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4.888580694717071</v>
+        <v>13.67729549471707</v>
       </c>
       <c r="C6" t="n">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -3662,15 +4458,34 @@
         </is>
       </c>
       <c r="B7" t="n">
+        <v>12.68327255575</v>
+      </c>
+      <c r="C7" t="n">
         <v>0</v>
       </c>
-      <c r="C7" t="n">
-        <v>50</v>
-      </c>
       <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ron</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="n">
+        <v>50</v>
+      </c>
+      <c r="D8" t="n">
         <v>1</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3685,7 +4500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3733,7 +4548,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>16.13594499959758</v>
+        <v>17.37632016338053</v>
       </c>
     </row>
     <row r="3">
@@ -3754,7 +4569,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>4.959627930598632</v>
+        <v>6.200003094381585</v>
       </c>
     </row>
     <row r="4">
@@ -3775,7 +4590,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>4.487152528116933</v>
+        <v>5.727527691899886</v>
       </c>
     </row>
     <row r="5">
@@ -3796,7 +4611,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>3.175570909293732</v>
+        <v>4.415946073076685</v>
       </c>
     </row>
     <row r="6">
@@ -3817,7 +4632,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>2.086755981054955</v>
+        <v>3.327131144837908</v>
       </c>
     </row>
     <row r="7">
@@ -3838,7 +4653,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>1.968795835707203</v>
+        <v>3.209170999490156</v>
       </c>
     </row>
     <row r="8">
@@ -3859,20 +4674,20 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>-0.8041534212441537</v>
+        <v>0.4362217425387991</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>eth</t>
+          <t>dot</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>6.427301587301571</v>
+        <v>6.618464956979999</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -3880,12 +4695,12 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>-1.237376466060306</v>
+        <v>0.1941620674010744</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -3893,7 +4708,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>5.235602094240846</v>
+        <v>6.427301587301571</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -3901,20 +4716,20 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>-2.429075959121031</v>
+        <v>0.002998697722646604</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ronin</t>
+          <t>axs</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>5.067611999999997</v>
+        <v>6.17283950824001</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -3922,20 +4737,20 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>-2.59706605336188</v>
+        <v>-0.2514633813389144</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>btc</t>
+          <t>eth</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>4.888580694717071</v>
+        <v>5.235602094240846</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -3943,20 +4758,20 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>-2.776097358644806</v>
+        <v>-1.188700795338078</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>uni</t>
+          <t>eth</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>4.574087329992842</v>
+        <v>5.195457959999999</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -3964,20 +4779,20 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>-3.090590723369035</v>
+        <v>-1.228844929578925</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>uni</t>
+          <t>ronin</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1.463680387409198</v>
+        <v>5.067611999999997</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -3985,20 +4800,20 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>-6.200997665952679</v>
+        <v>-1.356690889578927</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ronin</t>
+          <t>dot</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1.041666666666671</v>
+        <v>5.059132720920005</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -4006,28 +4821,217 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>-6.623011386695206</v>
+        <v>-1.365170168658919</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
+        <v>21</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>btc</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>4.888580694717071</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>-1.535722194861854</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>19</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>btc</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>4.817593600000002</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>-1.606709289578922</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>9</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>uni</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>4.574087329992842</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>-1.850215559586082</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>27</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>axs</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>4.491978610769991</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>-1.932324278808934</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>btc</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>3.971121199999999</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>-2.453181689578925</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>25</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>axs</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>2.018454436740001</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>-4.405848452838923</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>10</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>uni</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1.463680387409198</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>-4.960622502169726</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>7</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ronin</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1.041666666666671</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>-5.382636222912254</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ronin</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>0.8680555558159995</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>-5.556247333762925</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
         <v>8</v>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>uni</t>
         </is>
       </c>
-      <c r="C16" t="n">
+      <c r="C25" t="n">
         <v>0.609198903441964</v>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>PEOR TRADE</t>
         </is>
       </c>
-      <c r="E16" t="n">
-        <v>-7.055479149919913</v>
+      <c r="E25" t="n">
+        <v>-5.81510398613696</v>
       </c>
     </row>
   </sheetData>
@@ -4041,7 +5045,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M41"/>
+  <dimension ref="A1:M54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6131,6 +7135,697 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>16-07-2026 12:44:57</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>VENTA</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>16</v>
+      </c>
+      <c r="D42" t="n">
+        <v>17</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>btc</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>16-07-2026</t>
+        </is>
+      </c>
+      <c r="G42" s="1" t="inlineStr">
+        <is>
+          <t>0.00077259</t>
+        </is>
+      </c>
+      <c r="H42" t="n">
+        <v>64680</v>
+      </c>
+      <c r="I42" t="n">
+        <v>49.9711212</v>
+      </c>
+      <c r="J42" t="n">
+        <v>46</v>
+      </c>
+      <c r="K42" t="n">
+        <v>3.971121199999999</v>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>Venta registrada. Cantidad restante: 0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>16-07-2026 12:45:52</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>VENTA</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>19</v>
+      </c>
+      <c r="D43" t="n">
+        <v>18</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>btc</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>16-07-2026</t>
+        </is>
+      </c>
+      <c r="G43" s="1" t="inlineStr">
+        <is>
+          <t>0.00084752</t>
+        </is>
+      </c>
+      <c r="H43" t="n">
+        <v>64680</v>
+      </c>
+      <c r="I43" t="n">
+        <v>54.8175936</v>
+      </c>
+      <c r="J43" t="n">
+        <v>50</v>
+      </c>
+      <c r="K43" t="n">
+        <v>4.817593600000002</v>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>Venta registrada. Cantidad restante: 0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>05-08-2026 13:07:13</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>COMPRA</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>25</v>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>axs</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>5-08-2026</t>
+        </is>
+      </c>
+      <c r="G44" s="1" t="inlineStr">
+        <is>
+          <t>57.67012687</t>
+        </is>
+      </c>
+      <c r="H44" t="n">
+        <v>0.867</v>
+      </c>
+      <c r="I44" t="n">
+        <v>50</v>
+      </c>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>Compra registrada</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>14-08-2026 10:56:30</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>COMPRA</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>26</v>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>dot</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>14-08-2026</t>
+        </is>
+      </c>
+      <c r="G45" s="1" t="inlineStr">
+        <is>
+          <t>65.70302234</t>
+        </is>
+      </c>
+      <c r="H45" t="n">
+        <v>0.761</v>
+      </c>
+      <c r="I45" t="n">
+        <v>50</v>
+      </c>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>Compra registrada</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>19-08-2026 22:38:57</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>VENTA</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>25</v>
+      </c>
+      <c r="D46" t="n">
+        <v>19</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>axs</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>19-08-2026</t>
+        </is>
+      </c>
+      <c r="G46" s="1" t="inlineStr">
+        <is>
+          <t>57.67012687</t>
+        </is>
+      </c>
+      <c r="H46" t="n">
+        <v>0.902</v>
+      </c>
+      <c r="I46" t="n">
+        <v>52.01845443674</v>
+      </c>
+      <c r="J46" t="n">
+        <v>50</v>
+      </c>
+      <c r="K46" t="n">
+        <v>2.018454436740001</v>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>Venta registrada. Cantidad restante: 0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>19-08-2026 22:39:36</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>VENTA</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
+        <v>20</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>eth</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>19-08-2026</t>
+        </is>
+      </c>
+      <c r="G47" s="1" t="inlineStr">
+        <is>
+          <t>0.04948046</t>
+        </is>
+      </c>
+      <c r="H47" t="n">
+        <v>2126</v>
+      </c>
+      <c r="I47" t="n">
+        <v>105.19545796</v>
+      </c>
+      <c r="J47" t="n">
+        <v>100</v>
+      </c>
+      <c r="K47" t="n">
+        <v>5.195457959999999</v>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>Venta registrada. Cantidad restante: 0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>20-08-2026 12:36:30</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>VENTA</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>26</v>
+      </c>
+      <c r="D48" t="n">
+        <v>21</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>dot</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>20-08-2026</t>
+        </is>
+      </c>
+      <c r="G48" s="1" t="inlineStr">
+        <is>
+          <t>65.70302234</t>
+        </is>
+      </c>
+      <c r="H48" t="n">
+        <v>0.838</v>
+      </c>
+      <c r="I48" t="n">
+        <v>55.05913272092</v>
+      </c>
+      <c r="J48" t="n">
+        <v>50</v>
+      </c>
+      <c r="K48" t="n">
+        <v>5.059132720920005</v>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>Venta registrada. Cantidad restante: 0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>21-08-2026 12:39:04</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>VENTA</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>23</v>
+      </c>
+      <c r="D49" t="n">
+        <v>22</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>ronin</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>21-08-2026</t>
+        </is>
+      </c>
+      <c r="G49" s="1" t="inlineStr">
+        <is>
+          <t>868.05555556</t>
+        </is>
+      </c>
+      <c r="H49" t="n">
+        <v>0.0586</v>
+      </c>
+      <c r="I49" t="n">
+        <v>50.868055555816</v>
+      </c>
+      <c r="J49" t="n">
+        <v>50</v>
+      </c>
+      <c r="K49" t="n">
+        <v>0.8680555558159995</v>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>Venta registrada. Cantidad restante: 0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>22-08-2026 01:27:36</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>VENTA</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>24</v>
+      </c>
+      <c r="D50" t="n">
+        <v>23</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>axs</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>22-08-2026</t>
+        </is>
+      </c>
+      <c r="G50" s="1" t="inlineStr">
+        <is>
+          <t>51.44032922</t>
+        </is>
+      </c>
+      <c r="H50" t="n">
+        <v>1.092</v>
+      </c>
+      <c r="I50" t="n">
+        <v>56.17283950824001</v>
+      </c>
+      <c r="J50" t="n">
+        <v>50</v>
+      </c>
+      <c r="K50" t="n">
+        <v>6.17283950824001</v>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>Venta registrada. Cantidad restante: 0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>22-08-2026 01:30:42</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>VENTA</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>13</v>
+      </c>
+      <c r="D51" t="n">
+        <v>24</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>dot</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>22-08-2026</t>
+        </is>
+      </c>
+      <c r="G51" s="1" t="inlineStr">
+        <is>
+          <t>55.61735261</t>
+        </is>
+      </c>
+      <c r="H51" t="n">
+        <v>1.018</v>
+      </c>
+      <c r="I51" t="n">
+        <v>56.61846495698</v>
+      </c>
+      <c r="J51" t="n">
+        <v>50</v>
+      </c>
+      <c r="K51" t="n">
+        <v>6.618464956979999</v>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>Venta registrada. Cantidad restante: 0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>01-09-2026 11:39:28</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>COMPRA</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>27</v>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>axs</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>1-09-2026</t>
+        </is>
+      </c>
+      <c r="G52" s="1" t="inlineStr">
+        <is>
+          <t>53.47593583</t>
+        </is>
+      </c>
+      <c r="H52" t="n">
+        <v>0.9350000000000001</v>
+      </c>
+      <c r="I52" t="n">
+        <v>50</v>
+      </c>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>Compra registrada</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>16-09-2026 17:15:00</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>COMPRA</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>28</v>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>ron</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>19-09-2026</t>
+        </is>
+      </c>
+      <c r="G53" s="1" t="inlineStr">
+        <is>
+          <t>1057.08245243</t>
+        </is>
+      </c>
+      <c r="H53" t="n">
+        <v>0.0473</v>
+      </c>
+      <c r="I53" t="n">
+        <v>50</v>
+      </c>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>Compra registrada</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>18-09-2026 13:58:54</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>VENTA</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>27</v>
+      </c>
+      <c r="D54" t="n">
+        <v>25</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>axs</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>18-09-2026</t>
+        </is>
+      </c>
+      <c r="G54" s="1" t="inlineStr">
+        <is>
+          <t>53.47593583</t>
+        </is>
+      </c>
+      <c r="H54" t="n">
+        <v>1.019</v>
+      </c>
+      <c r="I54" t="n">
+        <v>54.49197861076999</v>
+      </c>
+      <c r="J54" t="n">
+        <v>50</v>
+      </c>
+      <c r="K54" t="n">
+        <v>4.491978610769991</v>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>Venta registrada. Cantidad restante: 0.0</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
actualizando ganancias y perdidas
</commit_message>
<xml_diff>
--- a/operaciones_crypto2.xlsx
+++ b/operaciones_crypto2.xlsx
@@ -948,17 +948,17 @@
       </c>
       <c r="G13" s="1" t="inlineStr">
         <is>
+          <t>846.02368866</t>
+        </is>
+      </c>
+      <c r="H13" s="1" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H13" s="1" t="inlineStr">
-        <is>
-          <t>846.02368866</t>
-        </is>
-      </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>CERRADA</t>
         </is>
       </c>
     </row>
@@ -1604,17 +1604,17 @@
       </c>
       <c r="G29" s="1" t="inlineStr">
         <is>
+          <t>1057.08245243</t>
+        </is>
+      </c>
+      <c r="H29" s="1" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H29" s="1" t="inlineStr">
-        <is>
-          <t>1057.08245243</t>
-        </is>
-      </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>CERRADA</t>
         </is>
       </c>
     </row>
@@ -1629,7 +1629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2552,6 +2552,76 @@
       </c>
       <c r="I26" t="n">
         <v>4.491978610769991</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="n">
+        <v>28</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ron</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>21-09-2026</t>
+        </is>
+      </c>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t>1057.08245243</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>0.0633</v>
+      </c>
+      <c r="G27" t="n">
+        <v>66.913319238819</v>
+      </c>
+      <c r="H27" t="n">
+        <v>50</v>
+      </c>
+      <c r="I27" t="n">
+        <v>16.913319238819</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="n">
+        <v>12</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ronin</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>21-09-2026</t>
+        </is>
+      </c>
+      <c r="E28" s="1" t="inlineStr">
+        <is>
+          <t>846.02368866</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>0.0633</v>
+      </c>
+      <c r="G28" t="n">
+        <v>53.55329949217799</v>
+      </c>
+      <c r="H28" t="n">
+        <v>50</v>
+      </c>
+      <c r="I28" t="n">
+        <v>3.553299492177992</v>
       </c>
     </row>
   </sheetData>
@@ -2565,7 +2635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2692,88 +2762,6 @@
         </is>
       </c>
       <c r="I3" t="inlineStr">
-        <is>
-          <t>ABIERTA</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>12</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>ronin</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>23-06-2026</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>50</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.0591</v>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>846.02368866</t>
-        </is>
-      </c>
-      <c r="G4" s="1" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H4" s="1" t="inlineStr">
-        <is>
-          <t>846.02368866</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>ABIERTA</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>28</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>ron</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>19-09-2026</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>50</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.0473</v>
-      </c>
-      <c r="F5" s="1" t="inlineStr">
-        <is>
-          <t>1057.08245243</t>
-        </is>
-      </c>
-      <c r="G5" s="1" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H5" s="1" t="inlineStr">
-        <is>
-          <t>1057.08245243</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
         <is>
           <t>ABIERTA</t>
         </is>
@@ -2790,7 +2778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N26"/>
+  <dimension ref="A1:N28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3447,11 +3435,11 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>dot</t>
+          <t>ronin</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -3461,29 +3449,29 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>22-08-2026</t>
+          <t>21-09-2026</t>
         </is>
       </c>
       <c r="E12" t="n">
         <v>50</v>
       </c>
       <c r="F12" t="n">
-        <v>56.61846495698</v>
+        <v>53.55329949217799</v>
       </c>
       <c r="G12" t="n">
-        <v>0.899</v>
+        <v>0.0591</v>
       </c>
       <c r="H12" t="n">
-        <v>1.018</v>
+        <v>0.0633</v>
       </c>
       <c r="I12" s="1" t="inlineStr">
         <is>
-          <t>55.61735261</t>
+          <t>846.02368866</t>
         </is>
       </c>
       <c r="J12" s="1" t="inlineStr">
         <is>
-          <t>55.61735261</t>
+          <t>846.02368866</t>
         </is>
       </c>
       <c r="K12" s="1" t="inlineStr">
@@ -3495,7 +3483,7 @@
         <v>50</v>
       </c>
       <c r="M12" t="n">
-        <v>6.618464956979999</v>
+        <v>3.553299492177992</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
@@ -3505,43 +3493,43 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>eth</t>
+          <t>dot</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>24-06-2026</t>
+          <t>23-06-2026</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>22-08-2026</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F13" t="n">
-        <v>112.6243059839605</v>
+        <v>56.61846495698</v>
       </c>
       <c r="G13" t="n">
-        <v>1621</v>
+        <v>0.899</v>
       </c>
       <c r="H13" t="n">
-        <v>1825.64</v>
+        <v>1.018</v>
       </c>
       <c r="I13" s="1" t="inlineStr">
         <is>
-          <t>0.06169031</t>
+          <t>55.61735261</t>
         </is>
       </c>
       <c r="J13" s="1" t="inlineStr">
         <is>
-          <t>0.06169031</t>
+          <t>55.61735261</t>
         </is>
       </c>
       <c r="K13" s="1" t="inlineStr">
@@ -3550,10 +3538,10 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="M13" t="n">
-        <v>12.62430598396051</v>
+        <v>6.618464956979999</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
@@ -3563,7 +3551,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -3572,34 +3560,34 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10-07-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F14" t="n">
-        <v>56.86052463211772</v>
+        <v>112.6243059839605</v>
       </c>
       <c r="G14" t="n">
-        <v>1563</v>
+        <v>1621</v>
       </c>
       <c r="H14" t="n">
-        <v>1777.46</v>
+        <v>1825.64</v>
       </c>
       <c r="I14" s="1" t="inlineStr">
         <is>
-          <t>0.03198976</t>
+          <t>0.06169031</t>
         </is>
       </c>
       <c r="J14" s="1" t="inlineStr">
         <is>
-          <t>0.03198976</t>
+          <t>0.06169031</t>
         </is>
       </c>
       <c r="K14" s="1" t="inlineStr">
@@ -3608,10 +3596,10 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="M14" t="n">
-        <v>6.860524632117723</v>
+        <v>12.62430598396051</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -3621,43 +3609,43 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>btc</t>
+          <t>eth</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>28-06-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>16-07-2026</t>
+          <t>10-07-2026</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F15" t="n">
-        <v>49.9711212</v>
+        <v>56.86052463211772</v>
       </c>
       <c r="G15" t="n">
-        <v>59540</v>
+        <v>1563</v>
       </c>
       <c r="H15" t="n">
-        <v>64680</v>
+        <v>1777.46</v>
       </c>
       <c r="I15" s="1" t="inlineStr">
         <is>
-          <t>0.00077259</t>
+          <t>0.03198976</t>
         </is>
       </c>
       <c r="J15" s="1" t="inlineStr">
         <is>
-          <t>0.00077259</t>
+          <t>0.03198976</t>
         </is>
       </c>
       <c r="K15" s="1" t="inlineStr">
@@ -3666,10 +3654,10 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="M15" t="n">
-        <v>3.971121199999999</v>
+        <v>6.860524632117723</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
@@ -3679,11 +3667,11 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>uni</t>
+          <t>btc</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -3693,29 +3681,29 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>10-07-2026</t>
+          <t>16-07-2026</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="F16" t="n">
-        <v>60.84024896265561</v>
+        <v>49.9711212</v>
       </c>
       <c r="G16" t="n">
-        <v>2.892</v>
+        <v>59540</v>
       </c>
       <c r="H16" t="n">
-        <v>3.519</v>
+        <v>64680</v>
       </c>
       <c r="I16" s="1" t="inlineStr">
         <is>
-          <t>17.28907331</t>
+          <t>0.00077259</t>
         </is>
       </c>
       <c r="J16" s="1" t="inlineStr">
         <is>
-          <t>17.28907331</t>
+          <t>0.00077259</t>
         </is>
       </c>
       <c r="K16" s="1" t="inlineStr">
@@ -3724,10 +3712,10 @@
         </is>
       </c>
       <c r="L16" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="M16" t="n">
-        <v>10.84024896265561</v>
+        <v>3.971121199999999</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
@@ -3737,7 +3725,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -3746,7 +3734,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>30-06-2026</t>
+          <t>28-06-2026</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -3758,22 +3746,22 @@
         <v>50</v>
       </c>
       <c r="F17" t="n">
-        <v>62.15183058147881</v>
+        <v>60.84024896265561</v>
       </c>
       <c r="G17" t="n">
-        <v>2.786</v>
+        <v>2.892</v>
       </c>
       <c r="H17" t="n">
-        <v>3.4631</v>
+        <v>3.519</v>
       </c>
       <c r="I17" s="1" t="inlineStr">
         <is>
-          <t>17.94687724</t>
+          <t>17.28907331</t>
         </is>
       </c>
       <c r="J17" s="1" t="inlineStr">
         <is>
-          <t>17.94687724</t>
+          <t>17.28907331</t>
         </is>
       </c>
       <c r="K17" s="1" t="inlineStr">
@@ -3785,7 +3773,7 @@
         <v>50</v>
       </c>
       <c r="M17" t="n">
-        <v>12.15183058147881</v>
+        <v>10.84024896265561</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
@@ -3795,11 +3783,11 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>btc</t>
+          <t>uni</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -3809,29 +3797,29 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>16-07-2026</t>
+          <t>10-07-2026</t>
         </is>
       </c>
       <c r="E18" t="n">
         <v>50</v>
       </c>
       <c r="F18" t="n">
-        <v>54.8175936</v>
+        <v>62.15183058147881</v>
       </c>
       <c r="G18" t="n">
-        <v>58996</v>
+        <v>2.786</v>
       </c>
       <c r="H18" t="n">
-        <v>64680</v>
+        <v>3.4631</v>
       </c>
       <c r="I18" s="1" t="inlineStr">
         <is>
-          <t>0.00084752</t>
+          <t>17.94687724</t>
         </is>
       </c>
       <c r="J18" s="1" t="inlineStr">
         <is>
-          <t>0.00084752</t>
+          <t>17.94687724</t>
         </is>
       </c>
       <c r="K18" s="1" t="inlineStr">
@@ -3843,7 +3831,7 @@
         <v>50</v>
       </c>
       <c r="M18" t="n">
-        <v>4.817593600000002</v>
+        <v>12.15183058147881</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
@@ -3853,11 +3841,11 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>eth</t>
+          <t>btc</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -3867,29 +3855,29 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>10-07-2026</t>
+          <t>16-07-2026</t>
         </is>
       </c>
       <c r="E19" t="n">
         <v>50</v>
       </c>
       <c r="F19" t="n">
-        <v>56.42730158730157</v>
+        <v>54.8175936</v>
       </c>
       <c r="G19" t="n">
-        <v>1575</v>
+        <v>58996</v>
       </c>
       <c r="H19" t="n">
-        <v>1777.46</v>
+        <v>64680</v>
       </c>
       <c r="I19" s="1" t="inlineStr">
         <is>
-          <t>0.03174603</t>
+          <t>0.00084752</t>
         </is>
       </c>
       <c r="J19" s="1" t="inlineStr">
         <is>
-          <t>0.03174603</t>
+          <t>0.00084752</t>
         </is>
       </c>
       <c r="K19" s="1" t="inlineStr">
@@ -3901,7 +3889,7 @@
         <v>50</v>
       </c>
       <c r="M19" t="n">
-        <v>6.427301587301571</v>
+        <v>4.817593600000002</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
@@ -3911,11 +3899,11 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>btc</t>
+          <t>eth</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3925,29 +3913,29 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>10-07-2026</t>
         </is>
       </c>
       <c r="E20" t="n">
         <v>50</v>
       </c>
       <c r="F20" t="n">
-        <v>54.88858069471707</v>
+        <v>56.42730158730157</v>
       </c>
       <c r="G20" t="n">
-        <v>58585</v>
+        <v>1575</v>
       </c>
       <c r="H20" t="n">
-        <v>64312.95</v>
+        <v>1777.46</v>
       </c>
       <c r="I20" s="1" t="inlineStr">
         <is>
-          <t>0.00085346</t>
+          <t>0.03174603</t>
         </is>
       </c>
       <c r="J20" s="1" t="inlineStr">
         <is>
-          <t>0.00085346</t>
+          <t>0.03174603</t>
         </is>
       </c>
       <c r="K20" s="1" t="inlineStr">
@@ -3959,7 +3947,7 @@
         <v>50</v>
       </c>
       <c r="M20" t="n">
-        <v>4.888580694717071</v>
+        <v>6.427301587301571</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
@@ -3969,11 +3957,11 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ronin</t>
+          <t>btc</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -3983,29 +3971,29 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>04-07-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="F21" t="n">
-        <v>47.067366</v>
+        <v>54.88858069471707</v>
       </c>
       <c r="G21" t="n">
-        <v>0.0547</v>
+        <v>58585</v>
       </c>
       <c r="H21" t="n">
-        <v>0.0613</v>
+        <v>64312.95</v>
       </c>
       <c r="I21" s="1" t="inlineStr">
         <is>
-          <t>767.82449726</t>
+          <t>0.00085346</t>
         </is>
       </c>
       <c r="J21" s="1" t="inlineStr">
         <is>
-          <t>767.82449726</t>
+          <t>0.00085346</t>
         </is>
       </c>
       <c r="K21" s="1" t="inlineStr">
@@ -4014,10 +4002,10 @@
         </is>
       </c>
       <c r="L21" t="n">
-        <v>41.999754</v>
+        <v>50</v>
       </c>
       <c r="M21" t="n">
-        <v>5.067611999999997</v>
+        <v>4.888580694717071</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
@@ -4027,7 +4015,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -4036,34 +4024,34 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>7-7-2026</t>
+          <t>30-06-2026</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>21-08-2026</t>
+          <t>04-07-2026</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="F22" t="n">
-        <v>50.868055555816</v>
+        <v>47.067366</v>
       </c>
       <c r="G22" t="n">
-        <v>0.0576</v>
+        <v>0.0547</v>
       </c>
       <c r="H22" t="n">
-        <v>0.0586</v>
+        <v>0.0613</v>
       </c>
       <c r="I22" s="1" t="inlineStr">
         <is>
-          <t>868.05555556</t>
+          <t>767.82449726</t>
         </is>
       </c>
       <c r="J22" s="1" t="inlineStr">
         <is>
-          <t>868.05555556</t>
+          <t>767.82449726</t>
         </is>
       </c>
       <c r="K22" s="1" t="inlineStr">
@@ -4072,10 +4060,10 @@
         </is>
       </c>
       <c r="L22" t="n">
-        <v>50</v>
+        <v>41.999754</v>
       </c>
       <c r="M22" t="n">
-        <v>0.8680555558159995</v>
+        <v>5.067611999999997</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
@@ -4085,43 +4073,43 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>axs</t>
+          <t>ronin</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>7-7-2026</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>22-08-2026</t>
+          <t>21-08-2026</t>
         </is>
       </c>
       <c r="E23" t="n">
         <v>50</v>
       </c>
       <c r="F23" t="n">
-        <v>56.17283950824001</v>
+        <v>50.868055555816</v>
       </c>
       <c r="G23" t="n">
-        <v>0.972</v>
+        <v>0.0576</v>
       </c>
       <c r="H23" t="n">
-        <v>1.092</v>
+        <v>0.0586</v>
       </c>
       <c r="I23" s="1" t="inlineStr">
         <is>
-          <t>51.44032922</t>
+          <t>868.05555556</t>
         </is>
       </c>
       <c r="J23" s="1" t="inlineStr">
         <is>
-          <t>51.44032922</t>
+          <t>868.05555556</t>
         </is>
       </c>
       <c r="K23" s="1" t="inlineStr">
@@ -4133,7 +4121,7 @@
         <v>50</v>
       </c>
       <c r="M23" t="n">
-        <v>6.17283950824001</v>
+        <v>0.8680555558159995</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
@@ -4143,7 +4131,7 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -4152,34 +4140,34 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>5-08-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>19-08-2026</t>
+          <t>22-08-2026</t>
         </is>
       </c>
       <c r="E24" t="n">
         <v>50</v>
       </c>
       <c r="F24" t="n">
-        <v>52.01845443674</v>
+        <v>56.17283950824001</v>
       </c>
       <c r="G24" t="n">
-        <v>0.867</v>
+        <v>0.972</v>
       </c>
       <c r="H24" t="n">
-        <v>0.902</v>
+        <v>1.092</v>
       </c>
       <c r="I24" s="1" t="inlineStr">
         <is>
-          <t>57.67012687</t>
+          <t>51.44032922</t>
         </is>
       </c>
       <c r="J24" s="1" t="inlineStr">
         <is>
-          <t>57.67012687</t>
+          <t>51.44032922</t>
         </is>
       </c>
       <c r="K24" s="1" t="inlineStr">
@@ -4191,7 +4179,7 @@
         <v>50</v>
       </c>
       <c r="M24" t="n">
-        <v>2.018454436740001</v>
+        <v>6.17283950824001</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
@@ -4201,43 +4189,43 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>dot</t>
+          <t>axs</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>14-08-2026</t>
+          <t>5-08-2026</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>20-08-2026</t>
+          <t>19-08-2026</t>
         </is>
       </c>
       <c r="E25" t="n">
         <v>50</v>
       </c>
       <c r="F25" t="n">
-        <v>55.05913272092</v>
+        <v>52.01845443674</v>
       </c>
       <c r="G25" t="n">
-        <v>0.761</v>
+        <v>0.867</v>
       </c>
       <c r="H25" t="n">
-        <v>0.838</v>
+        <v>0.902</v>
       </c>
       <c r="I25" s="1" t="inlineStr">
         <is>
-          <t>65.70302234</t>
+          <t>57.67012687</t>
         </is>
       </c>
       <c r="J25" s="1" t="inlineStr">
         <is>
-          <t>65.70302234</t>
+          <t>57.67012687</t>
         </is>
       </c>
       <c r="K25" s="1" t="inlineStr">
@@ -4249,7 +4237,7 @@
         <v>50</v>
       </c>
       <c r="M25" t="n">
-        <v>5.059132720920005</v>
+        <v>2.018454436740001</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
@@ -4259,57 +4247,173 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
+        <v>26</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>dot</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>14-08-2026</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>20-08-2026</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>50</v>
+      </c>
+      <c r="F26" t="n">
+        <v>55.05913272092</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.761</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.838</v>
+      </c>
+      <c r="I26" s="1" t="inlineStr">
+        <is>
+          <t>65.70302234</t>
+        </is>
+      </c>
+      <c r="J26" s="1" t="inlineStr">
+        <is>
+          <t>65.70302234</t>
+        </is>
+      </c>
+      <c r="K26" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L26" t="n">
+        <v>50</v>
+      </c>
+      <c r="M26" t="n">
+        <v>5.059132720920005</v>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
         <v>27</v>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>axs</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>1-09-2026</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>18-09-2026</t>
         </is>
       </c>
-      <c r="E26" t="n">
-        <v>50</v>
-      </c>
-      <c r="F26" t="n">
+      <c r="E27" t="n">
+        <v>50</v>
+      </c>
+      <c r="F27" t="n">
         <v>54.49197861076999</v>
       </c>
-      <c r="G26" t="n">
+      <c r="G27" t="n">
         <v>0.9350000000000001</v>
       </c>
-      <c r="H26" t="n">
+      <c r="H27" t="n">
         <v>1.019</v>
       </c>
-      <c r="I26" s="1" t="inlineStr">
+      <c r="I27" s="1" t="inlineStr">
         <is>
           <t>53.47593583</t>
         </is>
       </c>
-      <c r="J26" s="1" t="inlineStr">
+      <c r="J27" s="1" t="inlineStr">
         <is>
           <t>53.47593583</t>
         </is>
       </c>
-      <c r="K26" s="1" t="inlineStr">
+      <c r="K27" s="1" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L26" t="n">
-        <v>50</v>
-      </c>
-      <c r="M26" t="n">
+      <c r="L27" t="n">
+        <v>50</v>
+      </c>
+      <c r="M27" t="n">
         <v>4.491978610769991</v>
       </c>
-      <c r="N26" t="inlineStr">
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>28</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ron</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>19-09-2026</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>21-09-2026</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>50</v>
+      </c>
+      <c r="F28" t="n">
+        <v>66.913319238819</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0.0473</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0.0633</v>
+      </c>
+      <c r="I28" s="1" t="inlineStr">
+        <is>
+          <t>1057.08245243</t>
+        </is>
+      </c>
+      <c r="J28" s="1" t="inlineStr">
+        <is>
+          <t>1057.08245243</t>
+        </is>
+      </c>
+      <c r="K28" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L28" t="n">
+        <v>50</v>
+      </c>
+      <c r="M28" t="n">
+        <v>16.913319238819</v>
+      </c>
+      <c r="N28" t="inlineStr">
         <is>
           <t>CERRADA</t>
         </is>
@@ -4382,16 +4486,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6.977334222482668</v>
+        <v>10.53063371466066</v>
       </c>
       <c r="C3" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -4477,16 +4581,16 @@
         </is>
       </c>
       <c r="B8" t="n">
+        <v>16.913319238819</v>
+      </c>
+      <c r="C8" t="n">
         <v>0</v>
       </c>
-      <c r="C8" t="n">
-        <v>50</v>
-      </c>
       <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
         <v>1</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -4500,7 +4604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4548,20 +4652,20 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>17.37632016338053</v>
+        <v>17.08331966523287</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>eth</t>
+          <t>ron</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>12.62430598396051</v>
+        <v>16.913319238819</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -4569,20 +4673,20 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>6.200003094381585</v>
+        <v>10.19601585109242</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>uni</t>
+          <t>eth</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>12.15183058147881</v>
+        <v>12.62430598396051</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -4590,12 +4694,12 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>5.727527691899886</v>
+        <v>5.907002596233926</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -4603,7 +4707,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>10.84024896265561</v>
+        <v>12.15183058147881</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -4611,20 +4715,20 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>4.415946073076685</v>
+        <v>5.434527193752227</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>eth</t>
+          <t>uni</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>9.751434034416832</v>
+        <v>10.84024896265561</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -4632,20 +4736,20 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>3.327131144837908</v>
+        <v>4.122945574929026</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>uni</t>
+          <t>eth</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>9.63347388906908</v>
+        <v>9.751434034416832</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -4653,20 +4757,20 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>3.209170999490156</v>
+        <v>3.034130646690248</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>eth</t>
+          <t>uni</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>6.860524632117723</v>
+        <v>9.63347388906908</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -4674,20 +4778,20 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.4362217425387991</v>
+        <v>2.916170501342497</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>dot</t>
+          <t>eth</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>6.618464956979999</v>
+        <v>6.860524632117723</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -4695,20 +4799,20 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.1941620674010744</v>
+        <v>0.1432212443911398</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>eth</t>
+          <t>dot</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>6.427301587301571</v>
+        <v>6.618464956979999</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -4716,20 +4820,20 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.002998697722646604</v>
+        <v>-0.09883843074658483</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>axs</t>
+          <t>eth</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>6.17283950824001</v>
+        <v>6.427301587301571</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -4737,20 +4841,20 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>-0.2514633813389144</v>
+        <v>-0.2900018004250127</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>eth</t>
+          <t>axs</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>5.235602094240846</v>
+        <v>6.17283950824001</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -4758,12 +4862,12 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>-1.188700795338078</v>
+        <v>-0.5444638794865737</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -4771,7 +4875,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>5.195457959999999</v>
+        <v>5.235602094240846</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -4779,20 +4883,20 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>-1.228844929578925</v>
+        <v>-1.481701293485737</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ronin</t>
+          <t>eth</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>5.067611999999997</v>
+        <v>5.195457959999999</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -4800,20 +4904,20 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>-1.356690889578927</v>
+        <v>-1.521845427726585</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>dot</t>
+          <t>ronin</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>5.059132720920005</v>
+        <v>5.067611999999997</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -4821,20 +4925,20 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>-1.365170168658919</v>
+        <v>-1.649691387726587</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>btc</t>
+          <t>dot</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>4.888580694717071</v>
+        <v>5.059132720920005</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -4842,12 +4946,12 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>-1.535722194861854</v>
+        <v>-1.658170666806578</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -4855,7 +4959,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>4.817593600000002</v>
+        <v>4.888580694717071</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -4863,20 +4967,20 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>-1.606709289578922</v>
+        <v>-1.828722693009513</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>uni</t>
+          <t>btc</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>4.574087329992842</v>
+        <v>4.817593600000002</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -4884,20 +4988,20 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>-1.850215559586082</v>
+        <v>-1.899709787726581</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>axs</t>
+          <t>uni</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>4.491978610769991</v>
+        <v>4.574087329992842</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -4905,20 +5009,20 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>-1.932324278808934</v>
+        <v>-2.143216057733741</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>btc</t>
+          <t>axs</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>3.971121199999999</v>
+        <v>4.491978610769991</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -4926,20 +5030,20 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>-2.453181689578925</v>
+        <v>-2.225324776956593</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>axs</t>
+          <t>btc</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2.018454436740001</v>
+        <v>3.971121199999999</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -4947,20 +5051,20 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>-4.405848452838923</v>
+        <v>-2.746182187726585</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>uni</t>
+          <t>ronin</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1.463680387409198</v>
+        <v>3.553299492177992</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -4968,20 +5072,20 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>-4.960622502169726</v>
+        <v>-3.164003895548592</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ronin</t>
+          <t>axs</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1.041666666666671</v>
+        <v>2.018454436740001</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -4989,20 +5093,20 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>-5.382636222912254</v>
+        <v>-4.698848950986583</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ronin</t>
+          <t>uni</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.8680555558159995</v>
+        <v>1.463680387409198</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -5010,28 +5114,70 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>-5.556247333762925</v>
+        <v>-5.253623000317385</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
+        <v>7</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ronin</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1.041666666666671</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>-5.675636721059913</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ronin</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>0.8680555558159995</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>-5.849247831910584</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
         <v>8</v>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>uni</t>
         </is>
       </c>
-      <c r="C25" t="n">
+      <c r="C27" t="n">
         <v>0.609198903441964</v>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>PEOR TRADE</t>
         </is>
       </c>
-      <c r="E25" t="n">
-        <v>-5.81510398613696</v>
+      <c r="E27" t="n">
+        <v>-6.108104484284619</v>
       </c>
     </row>
   </sheetData>
@@ -5045,7 +5191,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M54"/>
+  <dimension ref="A1:M56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7826,6 +7972,116 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>21-09-2026 15:43:05</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>VENTA</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>28</v>
+      </c>
+      <c r="D55" t="n">
+        <v>26</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>ron</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>21-09-2026</t>
+        </is>
+      </c>
+      <c r="G55" s="1" t="inlineStr">
+        <is>
+          <t>1057.08245243</t>
+        </is>
+      </c>
+      <c r="H55" t="n">
+        <v>0.0633</v>
+      </c>
+      <c r="I55" t="n">
+        <v>66.913319238819</v>
+      </c>
+      <c r="J55" t="n">
+        <v>50</v>
+      </c>
+      <c r="K55" t="n">
+        <v>16.913319238819</v>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>Venta registrada. Cantidad restante: 0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>21-09-2026 15:48:38</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>VENTA</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>12</v>
+      </c>
+      <c r="D56" t="n">
+        <v>27</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>ronin</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>21-09-2026</t>
+        </is>
+      </c>
+      <c r="G56" s="1" t="inlineStr">
+        <is>
+          <t>846.02368866</t>
+        </is>
+      </c>
+      <c r="H56" t="n">
+        <v>0.0633</v>
+      </c>
+      <c r="I56" t="n">
+        <v>53.55329949217799</v>
+      </c>
+      <c r="J56" t="n">
+        <v>50</v>
+      </c>
+      <c r="K56" t="n">
+        <v>3.553299492177992</v>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>Venta registrada. Cantidad restante: 0.0</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>